<commit_message>
Protect all sheets in all 4 routine files with password
Every tab (Cómo funciona, Biblioteca, and the 4 routine sheets) is now
protected with the password. Cell lock states are preserved so users can
still edit the exercise dropdowns, the number of sets per exercise, and
the progress log, while formulas and structure stay locked.

https://claude.ai/code/session_013goGtNxneCGLBYieXpHUZd
</commit_message>
<xml_diff>
--- a/assets/rutinas-hombre-doble-progresion.xlsx
+++ b/assets/rutinas-hombre-doble-progresion.xlsx
@@ -9262,7 +9262,7 @@
     <row r="999" ht="15.75" customHeight="1" s="86"/>
     <row r="1000" ht="15.75" customHeight="1" s="86"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="de97"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="851A"/>
   <autoFilter ref="B4:F68"/>
   <mergeCells count="2">
     <mergeCell ref="B2:G2"/>
@@ -21312,7 +21312,7 @@
     <row r="999" ht="15.75" customHeight="1" s="86"/>
     <row r="1000" ht="15.75" customHeight="1" s="86"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="de97"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="851A"/>
   <mergeCells count="52">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="E24:F24"/>
@@ -36857,7 +36857,7 @@
     <row r="530" ht="15.75" customHeight="1" s="86"/>
     <row r="531" ht="15.75" customHeight="1" s="86"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="de97"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="851A"/>
   <mergeCells count="60">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="E24:F24"/>
@@ -54052,7 +54052,7 @@
     <row r="569" ht="15.75" customHeight="1" s="86"/>
     <row r="570" ht="15.75" customHeight="1" s="86"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="de97"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="851A"/>
   <mergeCells count="64">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="E24:F24"/>
@@ -73439,7 +73439,7 @@
     <row r="621" ht="15.75" customHeight="1" s="86"/>
     <row r="622" ht="15.75" customHeight="1" s="86"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="de97"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="851A"/>
   <mergeCells count="69">
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="B7:F7"/>

</xml_diff>